<commit_message>
Assignation des empreintes des composants de la première page
</commit_message>
<xml_diff>
--- a/Amplificateur_Audio/Amplificateur_Audio_Custom/Comparaison ref TI et Carte Custom.xlsx
+++ b/Amplificateur_Audio/Amplificateur_Audio_Custom/Comparaison ref TI et Carte Custom.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projet Kicad\Barre_de_Son_Dolby_DIY\Amplificateur_Audio\Amplificateur_Audio_Custom\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\le-ma\Documents\Projet electronique\Projet_Sound_Bar_DIY\Amplificateur_Audio\Amplificateur_Audio_Custom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{572BC3F3-E029-4B5F-B20B-6C5FCC8CC941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F4D474-D9D3-41AF-B895-2873E91B5675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FF8DD7E-34FE-43DF-B954-455528221A4E}"/>
+    <workbookView xWindow="3810" yWindow="1170" windowWidth="9620" windowHeight="12200" activeTab="1" xr2:uid="{4FF8DD7E-34FE-43DF-B954-455528221A4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Condensateur" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="172">
   <si>
     <t>Ref Ti</t>
   </si>
@@ -205,6 +205,354 @@
   </si>
   <si>
     <t>GRM155R71A104KA01D</t>
+  </si>
+  <si>
+    <t>33.2k</t>
+  </si>
+  <si>
+    <t>R38</t>
+  </si>
+  <si>
+    <t>R39</t>
+  </si>
+  <si>
+    <t>R40</t>
+  </si>
+  <si>
+    <t>R42</t>
+  </si>
+  <si>
+    <t>R44</t>
+  </si>
+  <si>
+    <t>R60</t>
+  </si>
+  <si>
+    <t>R61</t>
+  </si>
+  <si>
+    <t>R45</t>
+  </si>
+  <si>
+    <t>R201</t>
+  </si>
+  <si>
+    <t>R202</t>
+  </si>
+  <si>
+    <t>R203</t>
+  </si>
+  <si>
+    <t>R204</t>
+  </si>
+  <si>
+    <t>R205</t>
+  </si>
+  <si>
+    <t>R206</t>
+  </si>
+  <si>
+    <t>R207</t>
+  </si>
+  <si>
+    <t>R208</t>
+  </si>
+  <si>
+    <t>CRCW040233K2FKED</t>
+  </si>
+  <si>
+    <t>0402</t>
+  </si>
+  <si>
+    <t>2k</t>
+  </si>
+  <si>
+    <t>R235</t>
+  </si>
+  <si>
+    <t>R234</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>R13</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF2001X</t>
+  </si>
+  <si>
+    <t>R93</t>
+  </si>
+  <si>
+    <t>R94</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>100K</t>
+  </si>
+  <si>
+    <t>R64</t>
+  </si>
+  <si>
+    <t>0603</t>
+  </si>
+  <si>
+    <t>CRCW06030000Z0EA</t>
+  </si>
+  <si>
+    <t>R232</t>
+  </si>
+  <si>
+    <t>R231</t>
+  </si>
+  <si>
+    <t>R230</t>
+  </si>
+  <si>
+    <t>R233</t>
+  </si>
+  <si>
+    <t>CRCW0402100KFKED</t>
+  </si>
+  <si>
+    <t>47.5K</t>
+  </si>
+  <si>
+    <t>R41</t>
+  </si>
+  <si>
+    <t>R74</t>
+  </si>
+  <si>
+    <t>R229</t>
+  </si>
+  <si>
+    <t>R227</t>
+  </si>
+  <si>
+    <t>CRCW040247K5FKED</t>
+  </si>
+  <si>
+    <t>R228</t>
+  </si>
+  <si>
+    <t>R43</t>
+  </si>
+  <si>
+    <t>CRCW0402332RFKED</t>
+  </si>
+  <si>
+    <t>2.15K</t>
+  </si>
+  <si>
+    <t>R50</t>
+  </si>
+  <si>
+    <t>R63</t>
+  </si>
+  <si>
+    <t>R67</t>
+  </si>
+  <si>
+    <t>R69</t>
+  </si>
+  <si>
+    <t>R71</t>
+  </si>
+  <si>
+    <t>R73</t>
+  </si>
+  <si>
+    <t>R225</t>
+  </si>
+  <si>
+    <t>R224</t>
+  </si>
+  <si>
+    <t>R226</t>
+  </si>
+  <si>
+    <t>R223</t>
+  </si>
+  <si>
+    <t>R222</t>
+  </si>
+  <si>
+    <t>R221</t>
+  </si>
+  <si>
+    <t>CRCW04022K15FKED</t>
+  </si>
+  <si>
+    <t>R220</t>
+  </si>
+  <si>
+    <t>R216</t>
+  </si>
+  <si>
+    <t>R219</t>
+  </si>
+  <si>
+    <t>R218</t>
+  </si>
+  <si>
+    <t>R217</t>
+  </si>
+  <si>
+    <t>R215</t>
+  </si>
+  <si>
+    <t>R46</t>
+  </si>
+  <si>
+    <t>R62</t>
+  </si>
+  <si>
+    <t>R65</t>
+  </si>
+  <si>
+    <t>R68</t>
+  </si>
+  <si>
+    <t>R70</t>
+  </si>
+  <si>
+    <t>R72</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF1000X</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>R59</t>
+  </si>
+  <si>
+    <t>R54</t>
+  </si>
+  <si>
+    <t>R55</t>
+  </si>
+  <si>
+    <t>R56</t>
+  </si>
+  <si>
+    <t>R57</t>
+  </si>
+  <si>
+    <t>R58</t>
+  </si>
+  <si>
+    <t>R66</t>
+  </si>
+  <si>
+    <t>R209</t>
+  </si>
+  <si>
+    <t>R210</t>
+  </si>
+  <si>
+    <t>R211</t>
+  </si>
+  <si>
+    <t>R212</t>
+  </si>
+  <si>
+    <t>R213</t>
+  </si>
+  <si>
+    <t>R214</t>
+  </si>
+  <si>
+    <t>R236</t>
+  </si>
+  <si>
+    <t>CRCW040210K0FKED</t>
+  </si>
+  <si>
+    <t>CRCW060310K0FKEA</t>
+  </si>
+  <si>
+    <t>0602</t>
+  </si>
+  <si>
+    <t>2K</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>R11</t>
+  </si>
+  <si>
+    <t>R14</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>R16</t>
+  </si>
+  <si>
+    <t>R237</t>
+  </si>
+  <si>
+    <t>R238</t>
+  </si>
+  <si>
+    <t>R239</t>
+  </si>
+  <si>
+    <t>R240</t>
+  </si>
+  <si>
+    <t>R241</t>
+  </si>
+  <si>
+    <t>R242</t>
+  </si>
+  <si>
+    <t>R243</t>
+  </si>
+  <si>
+    <t>R244</t>
+  </si>
+  <si>
+    <t>R245</t>
+  </si>
+  <si>
+    <t>R246</t>
+  </si>
+  <si>
+    <t>R247</t>
+  </si>
+  <si>
+    <t>R248</t>
   </si>
 </sst>
 </file>
@@ -264,10 +612,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -588,14 +932,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A7B1A76-5DD3-4569-B12C-ED9F49EA38A1}">
   <dimension ref="A1:T34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.25" customWidth="1"/>
+    <col min="6" max="6" width="25.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -621,7 +965,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -659,7 +1003,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -681,7 +1025,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -694,7 +1038,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -707,7 +1051,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -720,7 +1064,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -733,7 +1077,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -746,7 +1090,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -759,7 +1103,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -788,7 +1132,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -844,7 +1188,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>39</v>
       </c>
@@ -882,7 +1226,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -917,7 +1261,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B29" s="3"/>
       <c r="D29" s="3"/>
       <c r="I29" s="3"/>
@@ -934,7 +1278,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B30" s="3"/>
       <c r="D30" s="3"/>
       <c r="I30" s="3"/>
@@ -951,7 +1295,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B31" s="3"/>
       <c r="D31" s="3"/>
       <c r="I31" s="3"/>
@@ -968,7 +1312,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B32" s="3"/>
       <c r="D32" s="3"/>
       <c r="I32" s="3"/>
@@ -985,7 +1329,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="33" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B33" s="3"/>
       <c r="D33" s="3"/>
       <c r="I33" s="3"/>
@@ -1002,7 +1346,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="34" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:19" x14ac:dyDescent="0.3">
       <c r="O34" t="s">
         <v>48</v>
       </c>
@@ -1025,9 +1369,1085 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D596A7B6-3493-4889-918C-0138A853E649}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:F111"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="10.6640625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="3">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="3"/>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="3"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="3"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="3"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="3"/>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="3">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1</v>
+      </c>
+      <c r="D24" s="3">
+        <v>2</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F24" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="3"/>
+      <c r="E25" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D26" s="3"/>
+      <c r="E26" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="3"/>
+      <c r="E27" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="3"/>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="3"/>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B30" s="3"/>
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B31" s="3"/>
+      <c r="D31" s="3"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="3">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" s="3">
+        <v>2</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" t="s">
+        <v>91</v>
+      </c>
+      <c r="D36" s="3"/>
+      <c r="E36" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B37" s="3"/>
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B38" s="3"/>
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B39" s="3"/>
+      <c r="D39" s="3"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B40" s="3"/>
+      <c r="D40" s="3"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B41" s="3"/>
+      <c r="D41" s="3"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B42" s="3"/>
+      <c r="D42" s="3"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>93</v>
+      </c>
+      <c r="B44" t="s">
+        <v>4</v>
+      </c>
+      <c r="D44" t="s">
+        <v>4</v>
+      </c>
+      <c r="F44" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B45" s="3">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1</v>
+      </c>
+      <c r="D45" s="3">
+        <v>2</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="3"/>
+      <c r="E46" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>95</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" t="s">
+        <v>97</v>
+      </c>
+      <c r="D47" s="3"/>
+      <c r="E47" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B48" s="3"/>
+      <c r="D48" s="3"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B49" s="3"/>
+      <c r="D49" s="3"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B50" s="3"/>
+      <c r="D50" s="3"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B51" s="3"/>
+      <c r="D51" s="3"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B52" s="3"/>
+      <c r="D52" s="3"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>332</v>
+      </c>
+      <c r="B55" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" t="s">
+        <v>4</v>
+      </c>
+      <c r="F55" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>0</v>
+      </c>
+      <c r="B56" s="3">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1</v>
+      </c>
+      <c r="D56" s="3">
+        <v>2</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F56" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>100</v>
+      </c>
+      <c r="B57" s="3"/>
+      <c r="C57" t="s">
+        <v>99</v>
+      </c>
+      <c r="D57" s="3"/>
+      <c r="E57" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B58" s="3"/>
+      <c r="D58" s="3"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B59" s="3"/>
+      <c r="D59" s="3"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B60" s="3"/>
+      <c r="D60" s="3"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B61" s="3"/>
+      <c r="D61" s="3"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B62" s="3"/>
+      <c r="D62" s="3"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B63" s="3"/>
+      <c r="D63" s="3"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>102</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4</v>
+      </c>
+      <c r="D65" t="s">
+        <v>4</v>
+      </c>
+      <c r="F65" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="3">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1</v>
+      </c>
+      <c r="D66" s="3">
+        <v>2</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F66" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>103</v>
+      </c>
+      <c r="B67" s="3"/>
+      <c r="C67" t="s">
+        <v>109</v>
+      </c>
+      <c r="D67" s="3"/>
+      <c r="E67" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>104</v>
+      </c>
+      <c r="B68" s="3"/>
+      <c r="C68" t="s">
+        <v>110</v>
+      </c>
+      <c r="D68" s="3"/>
+      <c r="E68" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>105</v>
+      </c>
+      <c r="B69" s="3"/>
+      <c r="C69" t="s">
+        <v>111</v>
+      </c>
+      <c r="D69" s="3"/>
+      <c r="E69" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>106</v>
+      </c>
+      <c r="B70" s="3"/>
+      <c r="C70" t="s">
+        <v>112</v>
+      </c>
+      <c r="D70" s="3"/>
+      <c r="E70" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>107</v>
+      </c>
+      <c r="B71" s="3"/>
+      <c r="C71" t="s">
+        <v>113</v>
+      </c>
+      <c r="D71" s="3"/>
+      <c r="E71" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>108</v>
+      </c>
+      <c r="B72" s="3"/>
+      <c r="C72" t="s">
+        <v>114</v>
+      </c>
+      <c r="D72" s="3"/>
+      <c r="E72" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B73" s="3"/>
+      <c r="D73" s="3"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>100</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4</v>
+      </c>
+      <c r="D77" t="s">
+        <v>4</v>
+      </c>
+      <c r="F77" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="3">
+        <v>1</v>
+      </c>
+      <c r="C78" t="s">
+        <v>1</v>
+      </c>
+      <c r="D78" s="3">
+        <v>2</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F78" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>122</v>
+      </c>
+      <c r="B79" s="3"/>
+      <c r="C79" t="s">
+        <v>116</v>
+      </c>
+      <c r="D79" s="3"/>
+      <c r="E79" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>123</v>
+      </c>
+      <c r="B80" s="3"/>
+      <c r="C80" t="s">
+        <v>117</v>
+      </c>
+      <c r="D80" s="3"/>
+      <c r="E80" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>124</v>
+      </c>
+      <c r="B81" s="3"/>
+      <c r="C81" t="s">
+        <v>118</v>
+      </c>
+      <c r="D81" s="3"/>
+      <c r="E81" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>125</v>
+      </c>
+      <c r="B82" s="3"/>
+      <c r="C82" t="s">
+        <v>119</v>
+      </c>
+      <c r="D82" s="3"/>
+      <c r="E82" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>126</v>
+      </c>
+      <c r="B83" s="3"/>
+      <c r="C83" t="s">
+        <v>120</v>
+      </c>
+      <c r="D83" s="3"/>
+      <c r="E83" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>127</v>
+      </c>
+      <c r="B84" s="3"/>
+      <c r="C84" t="s">
+        <v>121</v>
+      </c>
+      <c r="D84" s="3"/>
+      <c r="E84" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B85" s="3"/>
+      <c r="D85" s="3"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>129</v>
+      </c>
+      <c r="B88" t="s">
+        <v>4</v>
+      </c>
+      <c r="D88" t="s">
+        <v>4</v>
+      </c>
+      <c r="F88" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="3">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>1</v>
+      </c>
+      <c r="D89" s="3">
+        <v>2</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>130</v>
+      </c>
+      <c r="B90" s="3"/>
+      <c r="C90" t="s">
+        <v>137</v>
+      </c>
+      <c r="D90" s="3"/>
+      <c r="E90" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F90" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>131</v>
+      </c>
+      <c r="B91" s="3"/>
+      <c r="C91" t="s">
+        <v>138</v>
+      </c>
+      <c r="D91" s="3"/>
+      <c r="E91" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F91" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>132</v>
+      </c>
+      <c r="B92" s="3"/>
+      <c r="C92" t="s">
+        <v>139</v>
+      </c>
+      <c r="D92" s="3"/>
+      <c r="E92" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F92" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>133</v>
+      </c>
+      <c r="B93" s="3"/>
+      <c r="C93" t="s">
+        <v>140</v>
+      </c>
+      <c r="D93" s="3"/>
+      <c r="E93" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F93" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>134</v>
+      </c>
+      <c r="B94" s="3"/>
+      <c r="C94" t="s">
+        <v>141</v>
+      </c>
+      <c r="D94" s="3"/>
+      <c r="E94" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F94" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>135</v>
+      </c>
+      <c r="B95" s="3"/>
+      <c r="C95" t="s">
+        <v>142</v>
+      </c>
+      <c r="D95" s="3"/>
+      <c r="E95" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F95" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>136</v>
+      </c>
+      <c r="B96" s="3"/>
+      <c r="C96" t="s">
+        <v>143</v>
+      </c>
+      <c r="D96" s="3"/>
+      <c r="E96" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F96" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>147</v>
+      </c>
+      <c r="B98" t="s">
+        <v>4</v>
+      </c>
+      <c r="D98" t="s">
+        <v>4</v>
+      </c>
+      <c r="F98" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B99" s="3">
+        <v>1</v>
+      </c>
+      <c r="C99" t="s">
+        <v>1</v>
+      </c>
+      <c r="D99" s="3">
+        <v>2</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F99" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>148</v>
+      </c>
+      <c r="B100" s="3"/>
+      <c r="C100" t="s">
+        <v>160</v>
+      </c>
+      <c r="D100" s="3"/>
+      <c r="E100" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>149</v>
+      </c>
+      <c r="B101" s="3"/>
+      <c r="C101" t="s">
+        <v>161</v>
+      </c>
+      <c r="D101" s="3"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>150</v>
+      </c>
+      <c r="B102" s="3"/>
+      <c r="C102" t="s">
+        <v>162</v>
+      </c>
+      <c r="D102" s="3"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>151</v>
+      </c>
+      <c r="B103" s="3"/>
+      <c r="C103" t="s">
+        <v>163</v>
+      </c>
+      <c r="D103" s="3"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>152</v>
+      </c>
+      <c r="B104" s="3"/>
+      <c r="C104" t="s">
+        <v>164</v>
+      </c>
+      <c r="D104" s="3"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>153</v>
+      </c>
+      <c r="B105" s="3"/>
+      <c r="C105" t="s">
+        <v>165</v>
+      </c>
+      <c r="D105" s="3"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>154</v>
+      </c>
+      <c r="B106" s="3"/>
+      <c r="C106" t="s">
+        <v>166</v>
+      </c>
+      <c r="D106" s="3"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>155</v>
+      </c>
+      <c r="C107" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>156</v>
+      </c>
+      <c r="C108" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>157</v>
+      </c>
+      <c r="C109" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>158</v>
+      </c>
+      <c r="C110" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>159</v>
+      </c>
+      <c r="C111" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B99:B106"/>
+    <mergeCell ref="D99:D106"/>
+    <mergeCell ref="B66:B73"/>
+    <mergeCell ref="D66:D73"/>
+    <mergeCell ref="B78:B85"/>
+    <mergeCell ref="D78:D85"/>
+    <mergeCell ref="B89:B96"/>
+    <mergeCell ref="D89:D96"/>
+    <mergeCell ref="B35:B42"/>
+    <mergeCell ref="D35:D42"/>
+    <mergeCell ref="B45:B52"/>
+    <mergeCell ref="D45:D52"/>
+    <mergeCell ref="B56:B63"/>
+    <mergeCell ref="D56:D63"/>
+    <mergeCell ref="B2:B9"/>
+    <mergeCell ref="D2:D9"/>
+    <mergeCell ref="B14:B21"/>
+    <mergeCell ref="D14:D21"/>
+    <mergeCell ref="B24:B31"/>
+    <mergeCell ref="D24:D31"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout de point de test et début du routage
</commit_message>
<xml_diff>
--- a/Amplificateur_Audio/Amplificateur_Audio_Custom/Comparaison ref TI et Carte Custom.xlsx
+++ b/Amplificateur_Audio/Amplificateur_Audio_Custom/Comparaison ref TI et Carte Custom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projet Kicad\Barre_de_Son_Dolby_DIY\Amplificateur_Audio\Amplificateur_Audio_Custom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B436A2C-1AFE-48DA-9C8E-9769B52265EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26CBEB61-7393-4C3F-B46E-116E58614FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{4FF8DD7E-34FE-43DF-B954-455528221A4E}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{4FF8DD7E-34FE-43DF-B954-455528221A4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Condensateur" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="1297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2439" uniqueCount="1300">
   <si>
     <t>Ref Ti</t>
   </si>
@@ -3929,6 +3929,15 @@
   </si>
   <si>
     <t>Connector_PinHeader_2.54mm:PinHeader_2x25_P2.54mm_Vertical_SMD</t>
+  </si>
+  <si>
+    <t>EEV-FK1H102M</t>
+  </si>
+  <si>
+    <t>Capacitor_SMD:CP_Elec_16x17.5</t>
+  </si>
+  <si>
+    <t>F</t>
   </si>
 </sst>
 </file>
@@ -4016,7 +4025,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4045,7 +4054,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6607,7 +6615,7 @@
         <v>2</v>
       </c>
       <c r="F141" t="s">
-        <v>545</v>
+        <v>1297</v>
       </c>
       <c r="N141" t="s">
         <v>0</v>
@@ -6625,7 +6633,7 @@
         <v>2</v>
       </c>
       <c r="S141" t="s">
-        <v>545</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="142" spans="1:19">
@@ -6641,7 +6649,7 @@
         <v>1206</v>
       </c>
       <c r="F142" t="s">
-        <v>494</v>
+        <v>1298</v>
       </c>
       <c r="N142" t="s">
         <v>702</v>
@@ -6655,7 +6663,7 @@
         <v>1206</v>
       </c>
       <c r="S142" t="s">
-        <v>494</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="143" spans="1:19">
@@ -8834,15 +8842,6 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="379" spans="14:19">
-      <c r="N379" s="16"/>
-    </row>
-    <row r="380" spans="14:19">
-      <c r="N380" s="16"/>
-    </row>
-    <row r="381" spans="14:19">
-      <c r="N381" s="16"/>
-    </row>
     <row r="382" spans="14:19">
       <c r="N382" t="s">
         <v>3</v>
@@ -8883,9 +8882,6 @@
         <v>511</v>
       </c>
     </row>
-    <row r="385" spans="14:19">
-      <c r="N385" s="16"/>
-    </row>
     <row r="386" spans="14:19">
       <c r="N386" t="s">
         <v>414</v>
@@ -9147,6 +9143,78 @@
     </row>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="O169:O176"/>
+    <mergeCell ref="Q169:Q176"/>
+    <mergeCell ref="O141:O142"/>
+    <mergeCell ref="Q141:Q142"/>
+    <mergeCell ref="O147:O154"/>
+    <mergeCell ref="Q147:Q154"/>
+    <mergeCell ref="O158:O165"/>
+    <mergeCell ref="Q158:Q165"/>
+    <mergeCell ref="O121:O122"/>
+    <mergeCell ref="Q121:Q122"/>
+    <mergeCell ref="O125:O126"/>
+    <mergeCell ref="Q125:Q126"/>
+    <mergeCell ref="O131:O138"/>
+    <mergeCell ref="Q131:Q138"/>
+    <mergeCell ref="O95:O102"/>
+    <mergeCell ref="Q95:Q102"/>
+    <mergeCell ref="O105:O112"/>
+    <mergeCell ref="Q105:Q112"/>
+    <mergeCell ref="O115:O116"/>
+    <mergeCell ref="Q115:Q116"/>
+    <mergeCell ref="O73:O74"/>
+    <mergeCell ref="Q73:Q74"/>
+    <mergeCell ref="O79:O80"/>
+    <mergeCell ref="Q79:Q80"/>
+    <mergeCell ref="O84:O91"/>
+    <mergeCell ref="Q84:Q91"/>
+    <mergeCell ref="O44:O51"/>
+    <mergeCell ref="Q44:Q51"/>
+    <mergeCell ref="O55:O62"/>
+    <mergeCell ref="Q55:Q62"/>
+    <mergeCell ref="O67:O69"/>
+    <mergeCell ref="Q67:Q69"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="D79:D80"/>
+    <mergeCell ref="B44:B51"/>
+    <mergeCell ref="D44:D51"/>
+    <mergeCell ref="B55:B62"/>
+    <mergeCell ref="D55:D62"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="D73:D74"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="B29:B36"/>
+    <mergeCell ref="D29:D36"/>
+    <mergeCell ref="K15:K22"/>
+    <mergeCell ref="D2:D9"/>
+    <mergeCell ref="B2:B9"/>
+    <mergeCell ref="B15:B22"/>
+    <mergeCell ref="D15:D22"/>
+    <mergeCell ref="I15:I22"/>
+    <mergeCell ref="B84:B91"/>
+    <mergeCell ref="D84:D91"/>
+    <mergeCell ref="B95:B102"/>
+    <mergeCell ref="D95:D102"/>
+    <mergeCell ref="B105:B112"/>
+    <mergeCell ref="D105:D112"/>
+    <mergeCell ref="B115:B116"/>
+    <mergeCell ref="D115:D116"/>
+    <mergeCell ref="B121:B122"/>
+    <mergeCell ref="D121:D122"/>
+    <mergeCell ref="B125:B126"/>
+    <mergeCell ref="D125:D126"/>
+    <mergeCell ref="B158:B165"/>
+    <mergeCell ref="D158:D165"/>
+    <mergeCell ref="B169:B176"/>
+    <mergeCell ref="D169:D176"/>
+    <mergeCell ref="B131:B138"/>
+    <mergeCell ref="D131:D138"/>
+    <mergeCell ref="B141:B142"/>
+    <mergeCell ref="D141:D142"/>
+    <mergeCell ref="B147:B154"/>
+    <mergeCell ref="D147:D154"/>
     <mergeCell ref="O259:O266"/>
     <mergeCell ref="Q259:Q266"/>
     <mergeCell ref="O180:O187"/>
@@ -9159,78 +9227,6 @@
     <mergeCell ref="Q231:Q238"/>
     <mergeCell ref="Q248:Q255"/>
     <mergeCell ref="O248:O255"/>
-    <mergeCell ref="B158:B165"/>
-    <mergeCell ref="D158:D165"/>
-    <mergeCell ref="B169:B176"/>
-    <mergeCell ref="D169:D176"/>
-    <mergeCell ref="B131:B138"/>
-    <mergeCell ref="D131:D138"/>
-    <mergeCell ref="B141:B142"/>
-    <mergeCell ref="D141:D142"/>
-    <mergeCell ref="B147:B154"/>
-    <mergeCell ref="D147:D154"/>
-    <mergeCell ref="B115:B116"/>
-    <mergeCell ref="D115:D116"/>
-    <mergeCell ref="B121:B122"/>
-    <mergeCell ref="D121:D122"/>
-    <mergeCell ref="B125:B126"/>
-    <mergeCell ref="D125:D126"/>
-    <mergeCell ref="B84:B91"/>
-    <mergeCell ref="D84:D91"/>
-    <mergeCell ref="B95:B102"/>
-    <mergeCell ref="D95:D102"/>
-    <mergeCell ref="B105:B112"/>
-    <mergeCell ref="D105:D112"/>
-    <mergeCell ref="B29:B36"/>
-    <mergeCell ref="D29:D36"/>
-    <mergeCell ref="K15:K22"/>
-    <mergeCell ref="D2:D9"/>
-    <mergeCell ref="B2:B9"/>
-    <mergeCell ref="B15:B22"/>
-    <mergeCell ref="D15:D22"/>
-    <mergeCell ref="I15:I22"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="D79:D80"/>
-    <mergeCell ref="B44:B51"/>
-    <mergeCell ref="D44:D51"/>
-    <mergeCell ref="B55:B62"/>
-    <mergeCell ref="D55:D62"/>
-    <mergeCell ref="D67:D69"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="D73:D74"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="O44:O51"/>
-    <mergeCell ref="Q44:Q51"/>
-    <mergeCell ref="O55:O62"/>
-    <mergeCell ref="Q55:Q62"/>
-    <mergeCell ref="O67:O69"/>
-    <mergeCell ref="Q67:Q69"/>
-    <mergeCell ref="O73:O74"/>
-    <mergeCell ref="Q73:Q74"/>
-    <mergeCell ref="O79:O80"/>
-    <mergeCell ref="Q79:Q80"/>
-    <mergeCell ref="O84:O91"/>
-    <mergeCell ref="Q84:Q91"/>
-    <mergeCell ref="O95:O102"/>
-    <mergeCell ref="Q95:Q102"/>
-    <mergeCell ref="O105:O112"/>
-    <mergeCell ref="Q105:Q112"/>
-    <mergeCell ref="O115:O116"/>
-    <mergeCell ref="Q115:Q116"/>
-    <mergeCell ref="O121:O122"/>
-    <mergeCell ref="Q121:Q122"/>
-    <mergeCell ref="O125:O126"/>
-    <mergeCell ref="Q125:Q126"/>
-    <mergeCell ref="O131:O138"/>
-    <mergeCell ref="Q131:Q138"/>
-    <mergeCell ref="O169:O176"/>
-    <mergeCell ref="Q169:Q176"/>
-    <mergeCell ref="O141:O142"/>
-    <mergeCell ref="Q141:Q142"/>
-    <mergeCell ref="O147:O154"/>
-    <mergeCell ref="Q147:Q154"/>
-    <mergeCell ref="O158:O165"/>
-    <mergeCell ref="Q158:Q165"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10488,6 +10484,9 @@
       <c r="E71" s="2" t="s">
         <v>74</v>
       </c>
+      <c r="H71" t="s">
+        <v>1299</v>
+      </c>
       <c r="L71" s="15"/>
       <c r="N71" s="15"/>
       <c r="O71" s="2"/>
@@ -13325,12 +13324,26 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="L49:L51"/>
-    <mergeCell ref="N49:N51"/>
-    <mergeCell ref="N37:N39"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="L43:L45"/>
-    <mergeCell ref="N43:N45"/>
+    <mergeCell ref="L198:L200"/>
+    <mergeCell ref="N198:N200"/>
+    <mergeCell ref="L205:L207"/>
+    <mergeCell ref="N205:N207"/>
+    <mergeCell ref="L163:L165"/>
+    <mergeCell ref="N163:N165"/>
+    <mergeCell ref="L61:L63"/>
+    <mergeCell ref="N61:N63"/>
+    <mergeCell ref="L69:L71"/>
+    <mergeCell ref="N69:N71"/>
+    <mergeCell ref="L74:L76"/>
+    <mergeCell ref="N74:N76"/>
+    <mergeCell ref="B56:B63"/>
+    <mergeCell ref="D56:D63"/>
+    <mergeCell ref="B2:B9"/>
+    <mergeCell ref="D2:D9"/>
+    <mergeCell ref="B14:B21"/>
+    <mergeCell ref="D14:D21"/>
+    <mergeCell ref="B24:B31"/>
+    <mergeCell ref="D24:D31"/>
     <mergeCell ref="N2:N12"/>
     <mergeCell ref="L2:L12"/>
     <mergeCell ref="L15:L33"/>
@@ -13347,26 +13360,12 @@
     <mergeCell ref="D35:D42"/>
     <mergeCell ref="B45:B52"/>
     <mergeCell ref="D45:D52"/>
-    <mergeCell ref="B56:B63"/>
-    <mergeCell ref="D56:D63"/>
-    <mergeCell ref="B2:B9"/>
-    <mergeCell ref="D2:D9"/>
-    <mergeCell ref="B14:B21"/>
-    <mergeCell ref="D14:D21"/>
-    <mergeCell ref="B24:B31"/>
-    <mergeCell ref="D24:D31"/>
-    <mergeCell ref="L61:L63"/>
-    <mergeCell ref="N61:N63"/>
-    <mergeCell ref="L69:L71"/>
-    <mergeCell ref="N69:N71"/>
-    <mergeCell ref="L74:L76"/>
-    <mergeCell ref="N74:N76"/>
-    <mergeCell ref="L198:L200"/>
-    <mergeCell ref="N198:N200"/>
-    <mergeCell ref="L205:L207"/>
-    <mergeCell ref="N205:N207"/>
-    <mergeCell ref="L163:L165"/>
-    <mergeCell ref="N163:N165"/>
+    <mergeCell ref="L49:L51"/>
+    <mergeCell ref="N49:N51"/>
+    <mergeCell ref="N37:N39"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="L43:L45"/>
+    <mergeCell ref="N43:N45"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Modification d'empreinte et routage de sortie audio
</commit_message>
<xml_diff>
--- a/Amplificateur_Audio/Amplificateur_Audio_Custom/Comparaison ref TI et Carte Custom.xlsx
+++ b/Amplificateur_Audio/Amplificateur_Audio_Custom/Comparaison ref TI et Carte Custom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projet Kicad\Barre_de_Son_Dolby_DIY\Amplificateur_Audio\Amplificateur_Audio_Custom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26CBEB61-7393-4C3F-B46E-116E58614FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD18497-283C-48C9-B7EE-5F4BC143D635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{4FF8DD7E-34FE-43DF-B954-455528221A4E}"/>
+    <workbookView xWindow="-14505" yWindow="15" windowWidth="14610" windowHeight="15240" xr2:uid="{4FF8DD7E-34FE-43DF-B954-455528221A4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Condensateur" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2439" uniqueCount="1300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2439" uniqueCount="1302">
   <si>
     <t>Ref Ti</t>
   </si>
@@ -3938,6 +3938,12 @@
   </si>
   <si>
     <t>F</t>
+  </si>
+  <si>
+    <t>C409</t>
+  </si>
+  <si>
+    <t>CAP_EEVFK1H102M</t>
   </si>
 </sst>
 </file>
@@ -5286,7 +5292,7 @@
       </c>
       <c r="B59" s="15"/>
       <c r="C59" t="s">
-        <v>473</v>
+        <v>1300</v>
       </c>
       <c r="D59" s="15"/>
       <c r="N59" t="s">
@@ -6649,7 +6655,7 @@
         <v>1206</v>
       </c>
       <c r="F142" t="s">
-        <v>1298</v>
+        <v>1301</v>
       </c>
       <c r="N142" t="s">
         <v>702</v>

</xml_diff>